<commit_message>
Update Project Requirements Form (Excel).xlsx
</commit_message>
<xml_diff>
--- a/Project Requirements Form (Excel).xlsx
+++ b/Project Requirements Form (Excel).xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parke\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parke\OneDrive\Documents\GitHub\CodeTogether\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2E9DFFC-821E-4C6E-827A-C75BB8035C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F21791-C141-4848-9470-0C6C861ED7EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Requirements" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="141">
   <si>
     <t>CSCE 40003 Software Engineering</t>
   </si>
@@ -407,6 +407,48 @@
   </si>
   <si>
     <t>accurate forcasting</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>button works/ search works</t>
+  </si>
+  <si>
+    <t>launch</t>
+  </si>
+  <si>
+    <t>user can see,use and update home page</t>
+  </si>
+  <si>
+    <t>adding/removing music, playable, and audio works</t>
+  </si>
+  <si>
+    <t>enhanced experience at latest</t>
+  </si>
+  <si>
+    <t>list info for users to have an easier usage of functionality</t>
+  </si>
+  <si>
+    <t>pg can be viewed and update by users</t>
+  </si>
+  <si>
+    <t>user can see tips/frequently asked questions</t>
+  </si>
+  <si>
+    <t>user can use button to contact us</t>
+  </si>
+  <si>
+    <t>users can view and understand privacy policy page</t>
+  </si>
+  <si>
+    <t>visiable accurate date/time display</t>
+  </si>
+  <si>
+    <t>bday msg appears on appropriate day of users bday</t>
+  </si>
+  <si>
+    <t>messages appear and work correctly</t>
   </si>
 </sst>
 </file>
@@ -541,7 +583,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -579,6 +621,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1067,6 +1112,9 @@
       <c r="G11" s="2" t="s">
         <v>105</v>
       </c>
+      <c r="H11" s="2" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
@@ -1090,6 +1138,15 @@
       <c r="G12" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="H12" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
@@ -1113,6 +1170,9 @@
       <c r="G13" s="2" t="s">
         <v>105</v>
       </c>
+      <c r="H13" s="2" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
@@ -1136,6 +1196,15 @@
       <c r="G14" s="2" t="s">
         <v>105</v>
       </c>
+      <c r="H14" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
@@ -1177,7 +1246,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>8</v>
       </c>
@@ -1199,8 +1268,17 @@
       <c r="G17" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>9</v>
       </c>
@@ -1220,7 +1298,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>10</v>
       </c>
@@ -1237,7 +1315,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>11</v>
       </c>
@@ -1254,7 +1332,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>12</v>
       </c>
@@ -1274,7 +1352,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>13</v>
       </c>
@@ -1294,7 +1372,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>14</v>
       </c>
@@ -1311,7 +1389,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>15</v>
       </c>
@@ -1328,7 +1406,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>16</v>
       </c>
@@ -1345,7 +1423,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>17</v>
       </c>
@@ -1367,8 +1445,17 @@
       <c r="G26" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>18</v>
       </c>
@@ -1388,7 +1475,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>19</v>
       </c>
@@ -1407,8 +1494,17 @@
       <c r="G28" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H28" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>20</v>
       </c>
@@ -1425,7 +1521,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>21</v>
       </c>
@@ -1442,7 +1538,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>22</v>
       </c>
@@ -1459,7 +1555,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>23</v>
       </c>
@@ -1478,8 +1574,17 @@
       <c r="G32" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H32" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>24</v>
       </c>
@@ -1498,8 +1603,17 @@
       <c r="G33" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H33" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>25</v>
       </c>
@@ -1518,8 +1632,17 @@
       <c r="G34" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H34" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>26</v>
       </c>
@@ -1536,7 +1659,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>27</v>
       </c>
@@ -1555,8 +1678,17 @@
       <c r="G36" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H36" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>28</v>
       </c>
@@ -1578,8 +1710,17 @@
       <c r="G37" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H37" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>29</v>
       </c>
@@ -1598,8 +1739,17 @@
       <c r="G38" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H38" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>30</v>
       </c>
@@ -1616,7 +1766,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>31</v>
       </c>
@@ -1636,7 +1786,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>32</v>
       </c>
@@ -1653,21 +1803,21 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2"/>
     <row r="49" x14ac:dyDescent="0.2"/>
     <row r="50" x14ac:dyDescent="0.2"/>
     <row r="51" x14ac:dyDescent="0.2"/>

</xml_diff>